<commit_message>
[EDP-DDM-28147] Registry services requirements.
Change-Id: Ib1a33727e573f0bcbda223acc60eb60aba9e7292
</commit_message>
<xml_diff>
--- a/docs/ua/modules/arch/attachments/architecture/platform-system-requirements/registry-resources.xlsx
+++ b/docs/ua/modules/arch/attachments/architecture/platform-system-requirements/registry-resources.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Maksym_Kharchenko/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Maksym_Kharchenko/Work/Development/mdtu-ddm/mdtu-ddm-gerrit-workspace/mdtu-ddm/general/ddm-architecture/docs/ua/modules/arch/attachments/architecture/platform-system-requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0A9C770-4D25-9741-B108-599B8657515C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D966C3E-2F98-AA4E-8DB0-3BC59D58316C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{76BACE1B-BDCC-F34F-9205-7BB42BE8027F}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="47160" windowHeight="21580" xr2:uid="{76BACE1B-BDCC-F34F-9205-7BB42BE8027F}"/>
   </bookViews>
   <sheets>
     <sheet name="Registry Resources" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="110">
   <si>
     <t>Technology</t>
   </si>
@@ -314,39 +314,9 @@
     <t>Підсистема управління нереляційними базами даних</t>
   </si>
   <si>
-    <t>Service Mesh member</t>
-  </si>
-  <si>
     <t>Java</t>
   </si>
   <si>
-    <t>-Xms</t>
-  </si>
-  <si>
-    <t>-Xmx</t>
-  </si>
-  <si>
-    <t>1536m</t>
-  </si>
-  <si>
-    <t>768m</t>
-  </si>
-  <si>
-    <t>512m</t>
-  </si>
-  <si>
-    <t>1200m</t>
-  </si>
-  <si>
-    <t>128m</t>
-  </si>
-  <si>
-    <t>330m</t>
-  </si>
-  <si>
-    <t>?</t>
-  </si>
-  <si>
     <t>Type</t>
   </si>
   <si>
@@ -359,13 +329,43 @@
     <t>Zone</t>
   </si>
   <si>
-    <t>Criticality</t>
-  </si>
-  <si>
-    <t>non-critical</t>
-  </si>
-  <si>
-    <t>critical</t>
+    <t>Service Mesh</t>
+  </si>
+  <si>
+    <t>Monitoring</t>
+  </si>
+  <si>
+    <t>Java Opts</t>
+  </si>
+  <si>
+    <t>-XX:+ExplicitGCInvokesConcurrent -XX:+AlwaysPreTouch -XX:+UseG1GC</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -XX:+AlwaysPreTouch -XX:+UseG1GC</t>
+  </si>
+  <si>
+    <t>-Duser.timezone=UTC</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -Duser.timezone=UTC</t>
+  </si>
+  <si>
+    <t>-XX:+AlwaysPreTouch -XX:+UseG1GC</t>
+  </si>
+  <si>
+    <t>-Xms, Mb</t>
+  </si>
+  <si>
+    <t>-Xmx, Mb</t>
+  </si>
+  <si>
+    <t>-Xmn, Mb</t>
+  </si>
+  <si>
+    <t>Deployment Mode</t>
+  </si>
+  <si>
+    <t>Min Profile</t>
   </si>
 </sst>
 </file>
@@ -443,7 +443,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -452,11 +452,24 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -470,18 +483,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{06C99DE8-B980-0548-85E0-AAF92621FDD9}" name="Table3" displayName="Table3" ref="A1:I65" totalsRowShown="0">
-  <autoFilter ref="A1:I65" xr:uid="{06C99DE8-B980-0548-85E0-AAF92621FDD9}"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{06C99DE8-B980-0548-85E0-AAF92621FDD9}" name="Table3" displayName="Table3" ref="A1:M65" totalsRowShown="0">
+  <autoFilter ref="A1:M65" xr:uid="{06C99DE8-B980-0548-85E0-AAF92621FDD9}"/>
+  <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{7B40E2F0-02D6-904B-8018-66FABFA0DD1D}" name="Zone"/>
     <tableColumn id="2" xr3:uid="{9B6E3613-3147-0A49-A88D-DE5E5756377A}" name="Subsystem"/>
     <tableColumn id="3" xr3:uid="{7B693F86-BB20-4643-8C59-CE9AAFCBF004}" name="Component"/>
     <tableColumn id="4" xr3:uid="{BDC056D6-A828-3747-8D2F-B230006DB630}" name="Type"/>
-    <tableColumn id="9" xr3:uid="{26E395E2-1F19-C84B-980C-08C4B5582553}" name="Criticality"/>
-    <tableColumn id="5" xr3:uid="{E36D12C6-BEC1-3841-BB7F-07B8DD85B728}" name="Service Mesh member"/>
+    <tableColumn id="9" xr3:uid="{26E395E2-1F19-C84B-980C-08C4B5582553}" name="Deployment Mode"/>
+    <tableColumn id="14" xr3:uid="{206BB385-4C22-624D-A2DB-36D434439669}" name="Min Profile" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{E36D12C6-BEC1-3841-BB7F-07B8DD85B728}" name="Service Mesh" dataDxfId="0"/>
+    <tableColumn id="11" xr3:uid="{DE3293B1-99DC-3448-B36C-7DC56C231CB7}" name="Monitoring"/>
     <tableColumn id="6" xr3:uid="{90E59384-34DA-9D4D-8715-BED9DC803BBE}" name="Technology"/>
-    <tableColumn id="7" xr3:uid="{7D3E02CE-7CDD-5E44-88DF-1162888AE695}" name="-Xms"/>
-    <tableColumn id="8" xr3:uid="{3D28B649-AB9D-9C49-8889-6B0D4888A8D3}" name="-Xmx"/>
+    <tableColumn id="7" xr3:uid="{7D3E02CE-7CDD-5E44-88DF-1162888AE695}" name="-Xms, Mb"/>
+    <tableColumn id="8" xr3:uid="{3D28B649-AB9D-9C49-8889-6B0D4888A8D3}" name="-Xmx, Mb"/>
+    <tableColumn id="13" xr3:uid="{729BA2AA-0236-6D4E-88FA-AF5279155852}" name="-Xmn, Mb"/>
+    <tableColumn id="12" xr3:uid="{84FF7781-94A1-1246-98C1-52FEAF154639}" name="Java Opts"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -784,49 +801,64 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C809D083-7CF6-1445-A306-E810BD791428}">
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:M65"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="65.83203125" customWidth="1"/>
     <col min="3" max="3" width="35.5" customWidth="1"/>
     <col min="4" max="5" width="19.6640625" customWidth="1"/>
-    <col min="6" max="6" width="25" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" customWidth="1"/>
-    <col min="8" max="8" width="13.5" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" style="6" customWidth="1"/>
+    <col min="7" max="7" width="15.5" style="6" customWidth="1"/>
+    <col min="8" max="8" width="15.5" customWidth="1"/>
     <col min="9" max="9" width="14.33203125" customWidth="1"/>
+    <col min="10" max="10" width="13.5" customWidth="1"/>
+    <col min="11" max="12" width="14.33203125" customWidth="1"/>
+    <col min="13" max="13" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1" t="s">
+        <v>98</v>
+      </c>
+      <c r="I1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="K1" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B1" t="s">
-        <v>105</v>
-      </c>
-      <c r="C1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D1" t="s">
-        <v>103</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="L1" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="F1" t="s">
-        <v>92</v>
-      </c>
-      <c r="G1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>73</v>
       </c>
@@ -839,14 +871,14 @@
       <c r="D2" t="s">
         <v>15</v>
       </c>
-      <c r="E2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -859,14 +891,14 @@
       <c r="D3" t="s">
         <v>2</v>
       </c>
-      <c r="E3" t="s">
-        <v>108</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>73</v>
       </c>
@@ -879,14 +911,14 @@
       <c r="D4" t="s">
         <v>2</v>
       </c>
-      <c r="E4" t="s">
-        <v>108</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>73</v>
       </c>
@@ -899,14 +931,14 @@
       <c r="D5" t="s">
         <v>15</v>
       </c>
-      <c r="E5" t="s">
-        <v>108</v>
-      </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>73</v>
       </c>
@@ -919,23 +951,29 @@
       <c r="D6" t="s">
         <v>15</v>
       </c>
-      <c r="E6" t="s">
-        <v>108</v>
-      </c>
-      <c r="F6" t="s">
-        <v>3</v>
-      </c>
-      <c r="G6" t="s">
-        <v>93</v>
-      </c>
-      <c r="H6" t="s">
-        <v>102</v>
-      </c>
-      <c r="I6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F6" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>73</v>
       </c>
@@ -948,14 +986,14 @@
       <c r="D7" t="s">
         <v>15</v>
       </c>
-      <c r="E7" t="s">
-        <v>108</v>
-      </c>
-      <c r="F7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F7" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>73</v>
       </c>
@@ -968,14 +1006,14 @@
       <c r="D8" t="s">
         <v>15</v>
       </c>
-      <c r="E8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F8" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>73</v>
       </c>
@@ -988,14 +1026,14 @@
       <c r="D9" t="s">
         <v>15</v>
       </c>
-      <c r="E9" t="s">
-        <v>108</v>
-      </c>
-      <c r="F9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F9" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>73</v>
       </c>
@@ -1008,14 +1046,14 @@
       <c r="D10" t="s">
         <v>15</v>
       </c>
-      <c r="E10" t="s">
-        <v>108</v>
-      </c>
-      <c r="F10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>73</v>
       </c>
@@ -1028,23 +1066,29 @@
       <c r="D11" t="s">
         <v>15</v>
       </c>
-      <c r="E11" t="s">
-        <v>108</v>
-      </c>
-      <c r="F11" t="s">
-        <v>3</v>
-      </c>
-      <c r="G11" t="s">
-        <v>93</v>
-      </c>
-      <c r="H11" t="s">
-        <v>102</v>
-      </c>
-      <c r="I11" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F11" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>73</v>
       </c>
@@ -1057,14 +1101,29 @@
       <c r="D12" t="s">
         <v>15</v>
       </c>
-      <c r="E12" t="s">
-        <v>108</v>
-      </c>
-      <c r="F12" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F12" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="L12" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>73</v>
       </c>
@@ -1077,14 +1136,14 @@
       <c r="D13" t="s">
         <v>15</v>
       </c>
-      <c r="E13" t="s">
-        <v>108</v>
-      </c>
-      <c r="F13" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F13" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>73</v>
       </c>
@@ -1097,14 +1156,14 @@
       <c r="D14" t="s">
         <v>15</v>
       </c>
-      <c r="E14" t="s">
-        <v>108</v>
-      </c>
-      <c r="F14" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F14" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>73</v>
       </c>
@@ -1117,23 +1176,29 @@
       <c r="D15" t="s">
         <v>15</v>
       </c>
-      <c r="E15" t="s">
-        <v>108</v>
-      </c>
-      <c r="F15" t="s">
-        <v>9</v>
-      </c>
-      <c r="G15" t="s">
-        <v>93</v>
-      </c>
-      <c r="H15" t="s">
-        <v>98</v>
-      </c>
-      <c r="I15" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F15" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J15" s="6">
+        <v>512</v>
+      </c>
+      <c r="K15" s="6">
+        <v>512</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>73</v>
       </c>
@@ -1146,14 +1211,29 @@
       <c r="D16" t="s">
         <v>15</v>
       </c>
-      <c r="E16" t="s">
-        <v>108</v>
-      </c>
-      <c r="F16" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F16" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>73</v>
       </c>
@@ -1166,14 +1246,14 @@
       <c r="D17" t="s">
         <v>15</v>
       </c>
-      <c r="E17" t="s">
-        <v>108</v>
-      </c>
-      <c r="F17" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F17" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>74</v>
       </c>
@@ -1186,14 +1266,14 @@
       <c r="D18" t="s">
         <v>15</v>
       </c>
-      <c r="E18" t="s">
-        <v>109</v>
-      </c>
-      <c r="F18" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F18" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>74</v>
       </c>
@@ -1206,14 +1286,14 @@
       <c r="D19" t="s">
         <v>15</v>
       </c>
-      <c r="E19" t="s">
-        <v>109</v>
-      </c>
-      <c r="F19" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F19" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>74</v>
       </c>
@@ -1226,14 +1306,14 @@
       <c r="D20" t="s">
         <v>15</v>
       </c>
-      <c r="E20" t="s">
-        <v>109</v>
-      </c>
-      <c r="F20" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F20" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>74</v>
       </c>
@@ -1246,14 +1326,14 @@
       <c r="D21" t="s">
         <v>15</v>
       </c>
-      <c r="E21" t="s">
-        <v>109</v>
-      </c>
-      <c r="F21" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F21" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>74</v>
       </c>
@@ -1266,23 +1346,29 @@
       <c r="D22" t="s">
         <v>15</v>
       </c>
-      <c r="E22" t="s">
-        <v>109</v>
-      </c>
-      <c r="F22" t="s">
-        <v>3</v>
-      </c>
-      <c r="G22" t="s">
-        <v>93</v>
-      </c>
-      <c r="H22" t="s">
-        <v>96</v>
-      </c>
-      <c r="I22" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F22" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J22" s="6">
+        <v>1536</v>
+      </c>
+      <c r="K22" s="6">
+        <v>1536</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M22" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -1295,20 +1381,29 @@
       <c r="D23" t="s">
         <v>15</v>
       </c>
-      <c r="F23" t="s">
-        <v>3</v>
-      </c>
-      <c r="G23" t="s">
-        <v>93</v>
-      </c>
-      <c r="H23" t="s">
-        <v>98</v>
-      </c>
-      <c r="I23" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F23" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J23" s="6">
+        <v>512</v>
+      </c>
+      <c r="K23" s="6">
+        <v>512</v>
+      </c>
+      <c r="L23" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>74</v>
       </c>
@@ -1321,23 +1416,29 @@
       <c r="D24" t="s">
         <v>15</v>
       </c>
-      <c r="E24" t="s">
-        <v>109</v>
-      </c>
-      <c r="F24" t="s">
-        <v>3</v>
-      </c>
-      <c r="G24" t="s">
-        <v>93</v>
-      </c>
-      <c r="H24" t="s">
-        <v>102</v>
-      </c>
-      <c r="I24" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F24" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>74</v>
       </c>
@@ -1350,14 +1451,14 @@
       <c r="D25" t="s">
         <v>15</v>
       </c>
-      <c r="E25" t="s">
-        <v>109</v>
-      </c>
-      <c r="F25" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F25" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>74</v>
       </c>
@@ -1370,23 +1471,29 @@
       <c r="D26" t="s">
         <v>15</v>
       </c>
-      <c r="E26" t="s">
-        <v>109</v>
-      </c>
-      <c r="F26" t="s">
-        <v>3</v>
-      </c>
-      <c r="G26" t="s">
-        <v>93</v>
-      </c>
-      <c r="H26" t="s">
-        <v>101</v>
-      </c>
-      <c r="I26" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F26" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J26" s="6">
+        <v>330</v>
+      </c>
+      <c r="K26" s="6">
+        <v>330</v>
+      </c>
+      <c r="L26" s="6">
+        <v>200</v>
+      </c>
+      <c r="M26" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>74</v>
       </c>
@@ -1399,23 +1506,29 @@
       <c r="D27" t="s">
         <v>15</v>
       </c>
-      <c r="E27" t="s">
-        <v>109</v>
-      </c>
-      <c r="F27" t="s">
-        <v>3</v>
-      </c>
-      <c r="G27" t="s">
-        <v>93</v>
-      </c>
-      <c r="H27" t="s">
-        <v>101</v>
-      </c>
-      <c r="I27" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F27" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J27" s="6">
+        <v>330</v>
+      </c>
+      <c r="K27" s="6">
+        <v>330</v>
+      </c>
+      <c r="L27" s="6">
+        <v>200</v>
+      </c>
+      <c r="M27" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>74</v>
       </c>
@@ -1428,23 +1541,29 @@
       <c r="D28" t="s">
         <v>15</v>
       </c>
-      <c r="E28" t="s">
-        <v>109</v>
-      </c>
-      <c r="F28" t="s">
-        <v>3</v>
-      </c>
-      <c r="G28" t="s">
-        <v>93</v>
-      </c>
-      <c r="H28" t="s">
-        <v>98</v>
-      </c>
-      <c r="I28" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F28" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J28" s="6">
+        <v>512</v>
+      </c>
+      <c r="K28" s="6">
+        <v>512</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>74</v>
       </c>
@@ -1457,23 +1576,29 @@
       <c r="D29" t="s">
         <v>15</v>
       </c>
-      <c r="E29" t="s">
-        <v>109</v>
-      </c>
-      <c r="F29" t="s">
-        <v>3</v>
-      </c>
-      <c r="G29" t="s">
-        <v>93</v>
-      </c>
-      <c r="H29" t="s">
-        <v>98</v>
-      </c>
-      <c r="I29" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F29" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J29" s="6">
+        <v>512</v>
+      </c>
+      <c r="K29" s="6">
+        <v>512</v>
+      </c>
+      <c r="L29" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>74</v>
       </c>
@@ -1486,23 +1611,29 @@
       <c r="D30" t="s">
         <v>15</v>
       </c>
-      <c r="E30" t="s">
-        <v>109</v>
-      </c>
-      <c r="F30" t="s">
-        <v>3</v>
-      </c>
-      <c r="G30" t="s">
-        <v>93</v>
-      </c>
-      <c r="H30" t="s">
-        <v>99</v>
-      </c>
-      <c r="I30" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F30" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J30" s="6">
+        <v>1200</v>
+      </c>
+      <c r="K30" s="6">
+        <v>1200</v>
+      </c>
+      <c r="L30" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M30" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>74</v>
       </c>
@@ -1515,23 +1646,29 @@
       <c r="D31" t="s">
         <v>15</v>
       </c>
-      <c r="E31" t="s">
-        <v>109</v>
-      </c>
-      <c r="F31" t="s">
-        <v>3</v>
-      </c>
-      <c r="G31" t="s">
-        <v>93</v>
-      </c>
-      <c r="H31" t="s">
-        <v>99</v>
-      </c>
-      <c r="I31" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F31" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J31" s="6">
+        <v>1200</v>
+      </c>
+      <c r="K31" s="6">
+        <v>1200</v>
+      </c>
+      <c r="L31" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M31" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>74</v>
       </c>
@@ -1544,14 +1681,14 @@
       <c r="D32" t="s">
         <v>15</v>
       </c>
-      <c r="E32" t="s">
-        <v>109</v>
-      </c>
-      <c r="F32" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F32" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>74</v>
       </c>
@@ -1564,14 +1701,14 @@
       <c r="D33" t="s">
         <v>2</v>
       </c>
-      <c r="E33" t="s">
-        <v>109</v>
-      </c>
-      <c r="F33" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F33" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>74</v>
       </c>
@@ -1584,14 +1721,14 @@
       <c r="D34" t="s">
         <v>2</v>
       </c>
-      <c r="E34" t="s">
-        <v>109</v>
-      </c>
-      <c r="F34" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F34" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>74</v>
       </c>
@@ -1604,14 +1741,14 @@
       <c r="D35" t="s">
         <v>15</v>
       </c>
-      <c r="E35" t="s">
-        <v>109</v>
-      </c>
-      <c r="F35" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F35" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>74</v>
       </c>
@@ -1624,14 +1761,14 @@
       <c r="D36" t="s">
         <v>15</v>
       </c>
-      <c r="E36" t="s">
-        <v>109</v>
-      </c>
-      <c r="F36" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F36" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>74</v>
       </c>
@@ -1644,14 +1781,14 @@
       <c r="D37" t="s">
         <v>15</v>
       </c>
-      <c r="E37" t="s">
-        <v>109</v>
-      </c>
-      <c r="F37" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F37" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>74</v>
       </c>
@@ -1664,23 +1801,29 @@
       <c r="D38" t="s">
         <v>15</v>
       </c>
-      <c r="E38" t="s">
-        <v>109</v>
-      </c>
-      <c r="F38" t="s">
-        <v>3</v>
-      </c>
-      <c r="G38" t="s">
-        <v>93</v>
-      </c>
-      <c r="H38" t="s">
-        <v>98</v>
-      </c>
-      <c r="I38" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F38" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J38" s="6">
+        <v>512</v>
+      </c>
+      <c r="K38" s="6">
+        <v>512</v>
+      </c>
+      <c r="L38" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>74</v>
       </c>
@@ -1693,23 +1836,29 @@
       <c r="D39" t="s">
         <v>15</v>
       </c>
-      <c r="E39" t="s">
-        <v>109</v>
-      </c>
-      <c r="F39" t="s">
-        <v>3</v>
-      </c>
-      <c r="G39" t="s">
-        <v>93</v>
-      </c>
-      <c r="H39" t="s">
-        <v>101</v>
-      </c>
-      <c r="I39" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F39" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J39" s="6">
+        <v>330</v>
+      </c>
+      <c r="K39" s="6">
+        <v>330</v>
+      </c>
+      <c r="L39" s="6">
+        <v>200</v>
+      </c>
+      <c r="M39" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>74</v>
       </c>
@@ -1722,23 +1871,29 @@
       <c r="D40" t="s">
         <v>15</v>
       </c>
-      <c r="E40" t="s">
-        <v>109</v>
-      </c>
-      <c r="F40" t="s">
-        <v>3</v>
-      </c>
-      <c r="G40" t="s">
-        <v>93</v>
-      </c>
-      <c r="H40" t="s">
-        <v>99</v>
-      </c>
-      <c r="I40" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F40" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I40" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J40" s="6">
+        <v>1200</v>
+      </c>
+      <c r="K40" s="6">
+        <v>1200</v>
+      </c>
+      <c r="L40" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M40" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>74</v>
       </c>
@@ -1751,23 +1906,29 @@
       <c r="D41" t="s">
         <v>15</v>
       </c>
-      <c r="E41" t="s">
-        <v>109</v>
-      </c>
-      <c r="F41" t="s">
-        <v>3</v>
-      </c>
-      <c r="G41" t="s">
-        <v>93</v>
-      </c>
-      <c r="H41" t="s">
-        <v>99</v>
-      </c>
-      <c r="I41" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F41" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J41" s="6">
+        <v>1200</v>
+      </c>
+      <c r="K41" s="6">
+        <v>1200</v>
+      </c>
+      <c r="L41" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M41" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>74</v>
       </c>
@@ -1780,23 +1941,29 @@
       <c r="D42" t="s">
         <v>15</v>
       </c>
-      <c r="E42" t="s">
-        <v>109</v>
-      </c>
-      <c r="F42" t="s">
-        <v>3</v>
-      </c>
-      <c r="G42" t="s">
-        <v>93</v>
-      </c>
-      <c r="H42" t="s">
+      <c r="F42" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G42" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I42" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J42" s="6">
+        <v>128</v>
+      </c>
+      <c r="K42" s="6">
+        <v>128</v>
+      </c>
+      <c r="L42" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M42" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="I42" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>74</v>
       </c>
@@ -1809,14 +1976,29 @@
       <c r="D43" t="s">
         <v>15</v>
       </c>
-      <c r="E43" t="s">
-        <v>108</v>
-      </c>
-      <c r="F43" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F43" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="I43" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J43" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K43" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="L43" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>74</v>
       </c>
@@ -1829,23 +2011,29 @@
       <c r="D44" t="s">
         <v>15</v>
       </c>
-      <c r="E44" t="s">
-        <v>109</v>
-      </c>
-      <c r="F44" t="s">
-        <v>3</v>
-      </c>
-      <c r="G44" t="s">
-        <v>93</v>
-      </c>
-      <c r="H44" t="s">
-        <v>101</v>
-      </c>
-      <c r="I44" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F44" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J44" s="6">
+        <v>330</v>
+      </c>
+      <c r="K44" s="6">
+        <v>330</v>
+      </c>
+      <c r="L44" s="6">
+        <v>200</v>
+      </c>
+      <c r="M44" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>74</v>
       </c>
@@ -1858,23 +2046,29 @@
       <c r="D45" t="s">
         <v>15</v>
       </c>
-      <c r="E45" t="s">
-        <v>109</v>
-      </c>
-      <c r="F45" t="s">
-        <v>3</v>
-      </c>
-      <c r="G45" t="s">
-        <v>93</v>
-      </c>
-      <c r="H45" t="s">
+      <c r="F45" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I45" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J45" s="6">
+        <v>330</v>
+      </c>
+      <c r="K45" s="6">
+        <v>330</v>
+      </c>
+      <c r="L45" s="6">
+        <v>200</v>
+      </c>
+      <c r="M45" t="s">
         <v>101</v>
       </c>
-      <c r="I45" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>74</v>
       </c>
@@ -1887,23 +2081,29 @@
       <c r="D46" t="s">
         <v>15</v>
       </c>
-      <c r="E46" t="s">
-        <v>109</v>
-      </c>
-      <c r="F46" t="s">
-        <v>3</v>
-      </c>
-      <c r="G46" t="s">
-        <v>93</v>
-      </c>
-      <c r="H46" t="s">
+      <c r="F46" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I46" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J46" s="6">
+        <v>330</v>
+      </c>
+      <c r="K46" s="6">
+        <v>330</v>
+      </c>
+      <c r="L46" s="6">
+        <v>200</v>
+      </c>
+      <c r="M46" t="s">
         <v>101</v>
       </c>
-      <c r="I46" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>74</v>
       </c>
@@ -1916,23 +2116,29 @@
       <c r="D47" t="s">
         <v>15</v>
       </c>
-      <c r="E47" t="s">
-        <v>109</v>
-      </c>
-      <c r="F47" t="s">
-        <v>3</v>
-      </c>
-      <c r="G47" t="s">
-        <v>93</v>
-      </c>
-      <c r="H47" t="s">
+      <c r="F47" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G47" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I47" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J47" s="6">
+        <v>330</v>
+      </c>
+      <c r="K47" s="6">
+        <v>330</v>
+      </c>
+      <c r="L47" s="6">
+        <v>200</v>
+      </c>
+      <c r="M47" t="s">
         <v>101</v>
       </c>
-      <c r="I47" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>74</v>
       </c>
@@ -1945,23 +2151,29 @@
       <c r="D48" t="s">
         <v>15</v>
       </c>
-      <c r="E48" t="s">
-        <v>109</v>
-      </c>
-      <c r="F48" t="s">
-        <v>3</v>
-      </c>
-      <c r="G48" t="s">
-        <v>93</v>
-      </c>
-      <c r="H48" t="s">
-        <v>102</v>
-      </c>
-      <c r="I48" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F48" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G48" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I48" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J48" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K48" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="L48" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>74</v>
       </c>
@@ -1974,14 +2186,29 @@
       <c r="D49" t="s">
         <v>15</v>
       </c>
-      <c r="E49" t="s">
-        <v>109</v>
-      </c>
-      <c r="F49" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F49" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G49" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I49" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J49" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K49" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="L49" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>74</v>
       </c>
@@ -1994,14 +2221,14 @@
       <c r="D50" t="s">
         <v>15</v>
       </c>
-      <c r="E50" t="s">
-        <v>109</v>
-      </c>
-      <c r="F50" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F50" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G50" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>74</v>
       </c>
@@ -2014,14 +2241,14 @@
       <c r="D51" t="s">
         <v>15</v>
       </c>
-      <c r="E51" t="s">
-        <v>109</v>
-      </c>
-      <c r="F51" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F51" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G51" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>74</v>
       </c>
@@ -2034,23 +2261,29 @@
       <c r="D52" t="s">
         <v>15</v>
       </c>
-      <c r="E52" t="s">
-        <v>109</v>
-      </c>
-      <c r="F52" t="s">
-        <v>3</v>
-      </c>
-      <c r="G52" t="s">
-        <v>93</v>
-      </c>
-      <c r="H52" t="s">
+      <c r="F52" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I52" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J52" s="6">
+        <v>330</v>
+      </c>
+      <c r="K52" s="6">
+        <v>330</v>
+      </c>
+      <c r="L52" s="6">
+        <v>200</v>
+      </c>
+      <c r="M52" t="s">
         <v>101</v>
       </c>
-      <c r="I52" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>74</v>
       </c>
@@ -2063,23 +2296,29 @@
       <c r="D53" t="s">
         <v>15</v>
       </c>
-      <c r="E53" t="s">
-        <v>109</v>
-      </c>
-      <c r="F53" t="s">
-        <v>9</v>
-      </c>
-      <c r="G53" t="s">
-        <v>93</v>
-      </c>
-      <c r="H53" t="s">
-        <v>97</v>
+      <c r="F53" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G53" s="6" t="s">
+        <v>9</v>
       </c>
       <c r="I53" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+      <c r="J53" s="6">
+        <v>768</v>
+      </c>
+      <c r="K53" s="6">
+        <v>768</v>
+      </c>
+      <c r="L53" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M53" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>74</v>
       </c>
@@ -2092,14 +2331,14 @@
       <c r="D54" t="s">
         <v>2</v>
       </c>
-      <c r="E54" t="s">
-        <v>109</v>
-      </c>
-      <c r="F54" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F54" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G54" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>74</v>
       </c>
@@ -2112,14 +2351,14 @@
       <c r="D55" t="s">
         <v>15</v>
       </c>
-      <c r="E55" t="s">
-        <v>109</v>
-      </c>
-      <c r="F55" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F55" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G55" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>74</v>
       </c>
@@ -2132,14 +2371,14 @@
       <c r="D56" t="s">
         <v>15</v>
       </c>
-      <c r="E56" t="s">
-        <v>109</v>
-      </c>
-      <c r="F56" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F56" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G56" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>74</v>
       </c>
@@ -2152,14 +2391,14 @@
       <c r="D57" t="s">
         <v>2</v>
       </c>
-      <c r="E57" t="s">
-        <v>109</v>
-      </c>
-      <c r="F57" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F57" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G57" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>74</v>
       </c>
@@ -2172,14 +2411,14 @@
       <c r="D58" t="s">
         <v>2</v>
       </c>
-      <c r="E58" t="s">
-        <v>109</v>
-      </c>
-      <c r="F58" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F58" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G58" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>74</v>
       </c>
@@ -2192,14 +2431,14 @@
       <c r="D59" t="s">
         <v>15</v>
       </c>
-      <c r="E59" t="s">
-        <v>109</v>
-      </c>
-      <c r="F59" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F59" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>74</v>
       </c>
@@ -2212,14 +2451,14 @@
       <c r="D60" t="s">
         <v>15</v>
       </c>
-      <c r="E60" t="s">
-        <v>109</v>
-      </c>
-      <c r="F60" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F60" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G60" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>74</v>
       </c>
@@ -2232,14 +2471,14 @@
       <c r="D61" t="s">
         <v>2</v>
       </c>
-      <c r="E61" t="s">
-        <v>109</v>
-      </c>
-      <c r="F61" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F61" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G61" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>74</v>
       </c>
@@ -2252,14 +2491,14 @@
       <c r="D62" t="s">
         <v>2</v>
       </c>
-      <c r="E62" t="s">
-        <v>109</v>
-      </c>
-      <c r="F62" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F62" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G62" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>74</v>
       </c>
@@ -2272,14 +2511,14 @@
       <c r="D63" t="s">
         <v>15</v>
       </c>
-      <c r="E63" t="s">
-        <v>109</v>
-      </c>
-      <c r="F63" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F63" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G63" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>74</v>
       </c>
@@ -2292,14 +2531,14 @@
       <c r="D64" t="s">
         <v>2</v>
       </c>
-      <c r="E64" t="s">
-        <v>109</v>
-      </c>
-      <c r="F64" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F64" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G64" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>74</v>
       </c>
@@ -2312,10 +2551,10 @@
       <c r="D65" t="s">
         <v>15</v>
       </c>
-      <c r="E65" t="s">
-        <v>109</v>
-      </c>
-      <c r="F65" t="s">
+      <c r="F65" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G65" s="6" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>